<commit_message>
scan: seg5 2026-08-10 15:53 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-08-10.xlsx
+++ b/output/full_scan/batch_seq6_2026-08-10.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:O78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -527,21 +527,21 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>6206</v>
+        <v>6183</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>飛捷</t>
+          <t>關貿</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
         <v/>
       </c>
       <c r="D2" s="2" t="n">
-        <v>781.4295398605429</v>
+        <v>759.0715295797295</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>158</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -552,13 +552,13 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>69.8519648258317</v>
+        <v>57.72972358501564</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>22.36509063639624</v>
+        <v>24.80649994338685</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>2.2429539860543</v>
+        <v>0.8393055552133863</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>0</v>
@@ -570,31 +570,31 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>3.356136910500504</v>
+        <v>0.0516142484460759</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, rsi_strong, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, kd_golden_cross, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>6183</v>
+        <v>6206</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>關貿</t>
+          <t>飛捷</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
         <v/>
       </c>
       <c r="D3" s="2" t="n">
-        <v>779.0715295797295</v>
+        <v>741.4295398605429</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>92.90000000000001</v>
+        <v>158</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -605,13 +605,13 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>57.72972358501564</v>
+        <v>69.8519648258317</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>24.80649994338685</v>
+        <v>22.36509063639624</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0.8393055552133863</v>
+        <v>2.2429539860543</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>0</v>
@@ -623,11 +623,11 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.0516142484460759</v>
+        <v>3.356136910500504</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, rsi_strong, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, kd_golden_cross, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>739.9007446685157</v>
+        <v>699.9007446685157</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>80</v>
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>694.298599291236</v>
+        <v>674.298599291236</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1040</v>
@@ -739,21 +739,21 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>6426</v>
+        <v>6423</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>統新</t>
+          <t>億而得-創</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>667.2407417551258</v>
+        <v>646.479123855205</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>217.5</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -764,16 +764,16 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>65.00891190168468</v>
+        <v>62.04457810321975</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>23.59125144904065</v>
+        <v>24.75648321415393</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>3.528340892861066</v>
+        <v>2.364080393908019</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>0</v>
@@ -782,31 +782,31 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>8.13280202667679</v>
+        <v>1.871420111893109</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>6423</v>
+        <v>6426</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>億而得-創</t>
+          <t>統新</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>646.479123855205</v>
+        <v>627.2407417551258</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>82.40000000000001</v>
+        <v>217.5</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -817,16 +817,16 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>62.04457810321975</v>
+        <v>65.00891190168468</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>24.75648321415393</v>
+        <v>23.59125144904065</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>2.364080393908019</v>
+        <v>3.528340892861066</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0</v>
@@ -835,31 +835,31 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.871420111893109</v>
+        <v>8.13280202667679</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6213</v>
+        <v>6174</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>聯茂</t>
+          <t>安碁</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>607.5732718092964</v>
+        <v>588.7947111834289</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>427.5</v>
+        <v>42.1</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -870,16 +870,16 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>68.17267535409505</v>
+        <v>42.64256723209201</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>21.01192449358658</v>
+        <v>27.08809261864932</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.939831190477381</v>
+        <v>0.6669427503235502</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>0</v>
@@ -888,31 +888,31 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>12.04988962019979</v>
+        <v>-0.2637432742458458</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6416</v>
+        <v>6213</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>瑞祺電通</t>
+          <t>聯茂</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>599.7392298105297</v>
+        <v>567.5732718092964</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>103.5</v>
+        <v>427.5</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>61.07306364228874</v>
+        <v>68.17267535409505</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>22.36052036738694</v>
+        <v>21.01192449358658</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.8541636234026162</v>
+        <v>0.939831190477381</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.4293684829413609</v>
+        <v>12.04988962019979</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6225</v>
+        <v>6416</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>天瀚</t>
+          <t>瑞祺電通</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>597.5305158178907</v>
+        <v>559.7392298105297</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>27.7</v>
+        <v>103.5</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,13 +976,13 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>63.86523044436224</v>
+        <v>61.07306364228874</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>14.97469433694032</v>
+        <v>22.36052036738694</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1.371576731818218</v>
+        <v>0.8541636234026162</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0</v>
@@ -994,31 +994,31 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.2549384159791399</v>
+        <v>0.4293684829413609</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>6174</v>
+        <v>6225</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>安碁</t>
+          <t>天瀚</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>588.7947111834289</v>
+        <v>557.5305158178907</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>42.1</v>
+        <v>27.7</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,16 +1029,16 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>42.64256723209201</v>
+        <v>63.86523044436224</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>27.08809261864932</v>
+        <v>14.97469433694032</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.6669427503235502</v>
+        <v>1.371576731818218</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
         <v>0</v>
@@ -1047,31 +1047,31 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.2637432742458458</v>
+        <v>0.2549384159791399</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>6165</v>
+        <v>6243</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>浪凡</t>
+          <t>迅杰</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>586.0837748536428</v>
+        <v>546.8279966440317</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>50.9</v>
+        <v>45.7</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,13 +1082,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>57.42647306499502</v>
+        <v>49.73499215487036</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>15.63548067020227</v>
+        <v>24.50252557516282</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0.4083774853642788</v>
+        <v>0.4275410613229602</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -1100,31 +1100,31 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.1674920369763979</v>
+        <v>-0.775992343674111</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>6414</v>
+        <v>6165</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>樺漢</t>
+          <t>浪凡</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>578.6962739065256</v>
+        <v>546.0837748536428</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>482</v>
+        <v>50.9</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>63.98893928656253</v>
+        <v>57.42647306499502</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>22.63266797071104</v>
+        <v>15.63548067020227</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0.5780998580566509</v>
+        <v>0.4083774853642788</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>0</v>
@@ -1153,31 +1153,31 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1.853520720826112</v>
+        <v>0.1674920369763979</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>6257</v>
+        <v>6173</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>矽格</t>
+          <t>信昌電</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>574.4171668524763</v>
+        <v>541.4106605656436</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>207.5</v>
+        <v>168.5</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1188,13 +1188,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>48.23670684236492</v>
+        <v>42.68472073119765</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>20.23025813225657</v>
+        <v>34.40595260796817</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>1.105316696941825</v>
+        <v>1.192593663939603</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>0</v>
@@ -1206,31 +1206,31 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.5372968428071516</v>
+        <v>2.050485919277733</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>6196</v>
+        <v>6414</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>帆宣</t>
+          <t>樺漢</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>550.7388291927062</v>
+        <v>538.6962739065256</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>507</v>
+        <v>482</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,13 +1241,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>48.94670338794104</v>
+        <v>63.98893928656253</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>18.17108286298426</v>
+        <v>22.63266797071104</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0.5649022304227247</v>
+        <v>0.5780998580566509</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.09659835150966239</v>
+        <v>1.853520720826112</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>6173</v>
+        <v>6257</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>信昌電</t>
+          <t>矽格</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>541.4106605656436</v>
+        <v>534.4171668524763</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>168.5</v>
+        <v>207.5</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,13 +1294,13 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>42.68472073119765</v>
+        <v>48.23670684236492</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>34.40595260796817</v>
+        <v>20.23025813225657</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>1.192593663939603</v>
+        <v>1.105316696941825</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>0</v>
@@ -1312,31 +1312,31 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>2.050485919277733</v>
+        <v>0.5372968428071516</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>6191</v>
+        <v>6196</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>精成科</t>
+          <t>帆宣</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>526.5213487682032</v>
+        <v>510.7388291927062</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>87.2</v>
+        <v>507</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,13 +1347,13 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46.10082338888115</v>
+        <v>48.94670338794104</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>32.47729147557256</v>
+        <v>18.17108286298426</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0.9069630681754032</v>
+        <v>0.5649022304227247</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>0</v>
@@ -1365,31 +1365,31 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.3827828243389604</v>
+        <v>0.09659835150966239</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>6243</v>
+        <v>6207</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>迅杰</t>
+          <t>雷科</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>516.8279966440317</v>
+        <v>493.1233910795527</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45.7</v>
+        <v>107</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1400,16 +1400,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>49.73499215487036</v>
+        <v>45.35352010472476</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>24.50252557516282</v>
+        <v>24.01990798366345</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0.4275410613229602</v>
+        <v>0.8414466540819895</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L18" s="2" t="n">
         <v>0</v>
@@ -1418,31 +1418,31 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.775992343674111</v>
+        <v>0.0129623380944003</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>6192</v>
+        <v>6191</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>巨路</t>
+          <t>精成科</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>512.8844005003289</v>
+        <v>486.5213487682032</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>116</v>
+        <v>87.2</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1453,13 +1453,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>50.71970970820144</v>
+        <v>46.10082338888115</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>27.63184573698078</v>
+        <v>32.47729147557256</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>1.803305208082017</v>
+        <v>0.9069630681754032</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>0</v>
@@ -1471,31 +1471,31 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.6284810867254307</v>
+        <v>0.3827828243389604</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>6226</v>
+        <v>6188</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>光鼎</t>
+          <t>廣明</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>511.1181302095761</v>
+        <v>474.8406128108113</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>21.4</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,16 +1506,16 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>51.85707165608408</v>
+        <v>49.80207136706857</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>21.64916109257221</v>
+        <v>25.52727840673741</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>0.7261193329042747</v>
+        <v>0.5760718298255886</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>0</v>
@@ -1524,31 +1524,31 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-0.0858684090367485</v>
+        <v>0.7769172661227373</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>6202</v>
+        <v>6192</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>盛群</t>
+          <t>巨路</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>508.6656967592002</v>
+        <v>472.8844005003289</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>63.8</v>
+        <v>116</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1559,13 +1559,13 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>56.74697808965778</v>
+        <v>50.71970970820144</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>20.446544188162</v>
+        <v>27.63184573698078</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>0.7603994648675344</v>
+        <v>1.803305208082017</v>
       </c>
       <c r="K21" s="2" t="n">
         <v>0</v>
@@ -1577,31 +1577,31 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.117314594431419</v>
+        <v>0.6284810867254307</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>6214</v>
+        <v>6226</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>精誠</t>
+          <t>光鼎</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>505.1093242918259</v>
+        <v>471.1181302095761</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>144.5</v>
+        <v>21.4</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,13 +1612,13 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>51.90361828462773</v>
+        <v>51.85707165608408</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>13.55674118232764</v>
+        <v>21.64916109257221</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0.7395676640936464</v>
+        <v>0.7261193329042747</v>
       </c>
       <c r="K22" s="2" t="n">
         <v>0</v>
@@ -1630,31 +1630,31 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-0.0686585128964987</v>
+        <v>-0.0858684090367485</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>6207</v>
+        <v>6202</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>雷科</t>
+          <t>盛群</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>493.1233910795527</v>
+        <v>468.6656967592002</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>107</v>
+        <v>63.8</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,16 +1665,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>45.35352010472476</v>
+        <v>56.74697808965778</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>24.01990798366345</v>
+        <v>20.446544188162</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>0.8414466540819895</v>
+        <v>0.7603994648675344</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.0129623380944003</v>
+        <v>1.117314594431419</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>6188</v>
+        <v>6269</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>廣明</t>
+          <t>台郡</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>474.8406128108113</v>
+        <v>467.3790662214192</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>72.09999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>49.80207136706857</v>
+        <v>59.06299385342777</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>25.52727840673741</v>
+        <v>23.02567040809344</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.5760718298255886</v>
+        <v>1.755810145246609</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.7769172661227373</v>
+        <v>2.098634061476899</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>6269</v>
+        <v>6214</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>台郡</t>
+          <t>精誠</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>467.3790662214192</v>
+        <v>465.1093242918259</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>65.90000000000001</v>
+        <v>144.5</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,13 +1771,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>59.06299385342777</v>
+        <v>51.90361828462773</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>23.02567040809344</v>
+        <v>13.55674118232764</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>1.755810145246609</v>
+        <v>0.7395676640936464</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>2.098634061476899</v>
+        <v>-0.0686585128964987</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>6215</v>
+        <v>6204</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>和椿</t>
+          <t>艾華</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>444.0955443326735</v>
+        <v>434.4520395977325</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>102.5</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,13 +1824,13 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>54.4831845416134</v>
+        <v>49.38479745912756</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>20.62292992617979</v>
+        <v>32.70946694624664</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>1.618470111238015</v>
+        <v>2.159783213308927</v>
       </c>
       <c r="K26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.603861921628523</v>
+        <v>2.195641091635059</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6204</v>
+        <v>6456</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>艾華</t>
+          <t>GIS-KY</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>434.4520395977325</v>
+        <v>429.5605218768488</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>80.90000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,13 +1877,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>49.38479745912756</v>
+        <v>55.7413526864353</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>32.70946694624664</v>
+        <v>19.71368861988782</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>2.159783213308927</v>
+        <v>1.826702105975958</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>2.195641091635059</v>
+        <v>0.9622575759652472</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6451</v>
+        <v>6412</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>訊芯-KY</t>
+          <t>群電</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>432.1336928623746</v>
+        <v>426.4269401657284</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>456</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>51.91723260762927</v>
+        <v>43.0442641973437</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>20.75121944207835</v>
+        <v>32.45947676384331</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>1.17541246209539</v>
+        <v>0.6196459418887108</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>11.18580724096196</v>
+        <v>0.3570158784420925</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6282</v>
+        <v>6215</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>康舒</t>
+          <t>和椿</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>430.5686398964842</v>
+        <v>404.0955443326735</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>50</v>
+        <v>102.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,13 +1983,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>51.06184388891582</v>
+        <v>54.4831845416134</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>22.93307245830036</v>
+        <v>20.62292992617979</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>1.04928995115029</v>
+        <v>1.618470111238015</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.7979662344550689</v>
+        <v>1.603861921628523</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6164</v>
+        <v>6227</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>華興</t>
+          <t>茂綸</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>429.9545860402761</v>
+        <v>400.5733654378773</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>11.8</v>
+        <v>125</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,13 +2036,13 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>42.92545485830978</v>
+        <v>59.6060879416657</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>28.85861796316664</v>
+        <v>14.62738190139732</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.2785208213487328</v>
+        <v>0.7786837377881891</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.0073923597656112</v>
+        <v>1.726766377538268</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6412</v>
+        <v>6451</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>群電</t>
+          <t>訊芯-KY</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>426.4269401657284</v>
+        <v>392.1336928623746</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>79.40000000000001</v>
+        <v>456</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>43.0442641973437</v>
+        <v>51.91723260762927</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>32.45947676384331</v>
+        <v>20.75121944207835</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.6196459418887108</v>
+        <v>1.17541246209539</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.3570158784420925</v>
+        <v>11.18580724096196</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6271</v>
+        <v>6229</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>同欣電</t>
+          <t>研通</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>425.8236690474123</v>
+        <v>390.7053521503887</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>197</v>
+        <v>23.55</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,16 +2142,16 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>48.91352016282462</v>
+        <v>44.50445772105656</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>23.13023124621723</v>
+        <v>23.71939551545771</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.9825193022842416</v>
+        <v>0.2669724967060971</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>3.554357245802505</v>
+        <v>0.1581766699771224</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6168</v>
+        <v>6282</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>宏齊</t>
+          <t>康舒</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>405.5998715595856</v>
+        <v>390.5686398964842</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>25.05</v>
+        <v>50</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>50.14145864011715</v>
+        <v>51.06184388891582</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>21.92519634713251</v>
+        <v>22.93307245830036</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.920718696931504</v>
+        <v>1.04928995115029</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.3851070248310393</v>
+        <v>0.7979662344550689</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6456</v>
+        <v>6164</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>GIS-KY</t>
+          <t>華興</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>399.5605218768488</v>
+        <v>389.9545860402761</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>67.59999999999999</v>
+        <v>11.8</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,13 +2248,13 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>55.7413526864353</v>
+        <v>42.92545485830978</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>19.71368861988782</v>
+        <v>28.85861796316664</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1.826702105975958</v>
+        <v>0.2785208213487328</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.9622575759652472</v>
+        <v>0.0073923597656112</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6190</v>
+        <v>6271</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>萬泰科</t>
+          <t>同欣電</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>371.4921416834692</v>
+        <v>385.8236690474123</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>68.8</v>
+        <v>197</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>47.05627038961318</v>
+        <v>48.91352016282462</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>32.08947107167344</v>
+        <v>23.13023124621723</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.8270287635314424</v>
+        <v>0.9825193022842416</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.5251318219281336</v>
+        <v>3.554357245802505</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>6449</v>
+        <v>6168</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>鈺邦</t>
+          <t>宏齊</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>367.6955893517073</v>
+        <v>385.5998715595856</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>240.5</v>
+        <v>25.05</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,13 +2354,13 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>44.6919693221508</v>
+        <v>50.14145864011715</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>31.57261110678408</v>
+        <v>21.92519634713251</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.7398891102966632</v>
+        <v>0.920718696931504</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>4.239608341688111</v>
+        <v>0.3851070248310393</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>6224</v>
+        <v>6190</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>聚鼎</t>
+          <t>萬泰科</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>364.8592085479777</v>
+        <v>371.4921416834692</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>56</v>
+        <v>68.8</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,16 +2407,16 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>42.21910147936961</v>
+        <v>47.05627038961318</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>32.83834489354695</v>
+        <v>32.08947107167344</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.4784450780377132</v>
+        <v>0.8270287635314424</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.8945242461589924</v>
+        <v>0.5251318219281336</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>6166</v>
+        <v>6281</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>凌華</t>
+          <t>全國電</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>363.2439352713656</v>
+        <v>355.0187119470689</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>143</v>
+        <v>51.6</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>54.01399777908643</v>
+        <v>50.1666281495004</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>17.36199313882288</v>
+        <v>17.28403047352334</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.6056307244439875</v>
+        <v>0.5898495629800935</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.5420628163513347</v>
+        <v>-0.0431077101336801</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6281</v>
+        <v>6187</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>全國電</t>
+          <t>萬潤</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>355.0187119470689</v>
+        <v>354.5936112175816</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>51.6</v>
+        <v>1090</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,49 +2513,49 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>50.1666281495004</v>
+        <v>53.46111170044246</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>17.28403047352334</v>
+        <v>12.3087041217293</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.5898495629800935</v>
+        <v>1.514857326548334</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M39" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.0431077101336801</v>
+        <v>22.09232555567394</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6187</v>
+        <v>6175</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>萬潤</t>
+          <t>立敦</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>354.5936112175816</v>
+        <v>348.4476963018541</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>1090</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,49 +2566,49 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>53.46111170044246</v>
+        <v>38.72763810708439</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>12.3087041217293</v>
+        <v>25.87997541245723</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>1.514857326548334</v>
+        <v>0.3590619387938579</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>22.09232555567394</v>
+        <v>-0.0359591325848578</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6175</v>
+        <v>6194</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>立敦</t>
+          <t>育富</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>348.4476963018541</v>
+        <v>347.7573265565226</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>75.59999999999999</v>
+        <v>30</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,16 +2619,16 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>38.72763810708439</v>
+        <v>43.18199965040478</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>25.87997541245723</v>
+        <v>28.94073767614961</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.3590619387938579</v>
+        <v>0.7278523181695278</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.0359591325848578</v>
+        <v>0.0906848257259589</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6194</v>
+        <v>6163</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>育富</t>
+          <t>華電網</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>347.7573265565226</v>
+        <v>338.2535835834404</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,16 +2672,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>43.18199965040478</v>
+        <v>47.96628956233509</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>28.94073767614961</v>
+        <v>27.96189953778999</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.7278523181695278</v>
+        <v>0.42215608371619</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.0906848257259589</v>
+        <v>0.5647133368152435</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6285</v>
+        <v>6449</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>啟碁</t>
+          <t>鈺邦</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>344.6446341049075</v>
+        <v>327.6955893517073</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>256</v>
+        <v>240.5</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,13 +2725,13 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>53.1038400026636</v>
+        <v>44.6919693221508</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>19.05769318803712</v>
+        <v>31.57261110678408</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>1.288124327605217</v>
+        <v>0.7398891102966632</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>2.422875656530869</v>
+        <v>4.239608341688111</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6278</v>
+        <v>6224</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>台表科</t>
+          <t>聚鼎</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>338.6762966894772</v>
+        <v>324.8592085479777</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>171.5</v>
+        <v>56</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>52.11554347801326</v>
+        <v>42.21910147936961</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>28.39550416933267</v>
+        <v>32.83834489354695</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>1.535899867764819</v>
+        <v>0.4784450780377132</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>3.261276972419939</v>
+        <v>0.8945242461589924</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6163</v>
+        <v>6166</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>華電網</t>
+          <t>凌華</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>338.2535835834404</v>
+        <v>323.2439352713656</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>42</v>
+        <v>143</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,16 +2831,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>47.96628956233509</v>
+        <v>54.01399777908643</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>27.96189953778999</v>
+        <v>17.36199313882288</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.42215608371619</v>
+        <v>0.6056307244439875</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.5647133368152435</v>
+        <v>0.5420628163513347</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6197</v>
+        <v>6278</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>佳必琪</t>
+          <t>台表科</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>330.7420034366085</v>
+        <v>318.6762966894772</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>309</v>
+        <v>171.5</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>49.27257213589504</v>
+        <v>52.11554347801326</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>19.20985592526348</v>
+        <v>28.39550416933267</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.9648127531215788</v>
+        <v>1.535899867764819</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.9338417424029366</v>
+        <v>3.261276972419939</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6239</v>
+        <v>6477</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>安集</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>319.235622848787</v>
+        <v>316.4502613287738</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>288.5</v>
+        <v>33.95</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>52.97887863304339</v>
+        <v>43.37166705898985</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>16.93969890618489</v>
+        <v>16.97922797804473</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.3712256943201117</v>
+        <v>0.2215247056356196</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>3.553993633587414</v>
+        <v>-0.5107340494142445</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6442</v>
+        <v>6220</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>岳豐</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>295.8860407547625</v>
+        <v>309.8850668686963</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>1425</v>
+        <v>25.75</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>51.16117003979465</v>
+        <v>35.84961710887379</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>23.67396318234185</v>
+        <v>30.8699502661992</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1.204091036502204</v>
+        <v>0.7666573207713016</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>39.23105388440921</v>
+        <v>0.0596857528714043</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6208</v>
+        <v>6285</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>日揚</t>
+          <t>啟碁</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>291.3313815875944</v>
+        <v>304.6446341049075</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>81.7</v>
+        <v>256</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>44.02708707802903</v>
+        <v>53.1038400026636</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>16.66578478987826</v>
+        <v>19.05769318803712</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.9407008158382956</v>
+        <v>1.288124327605217</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.2488588667002425</v>
+        <v>2.422875656530869</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6272</v>
+        <v>6223</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>驊陞</t>
+          <t>旺矽</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>287.9809485687836</v>
+        <v>291.7388476456422</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>25.1</v>
+        <v>6225</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>39.49926573118158</v>
+        <v>53.77850832992098</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>40.31524748927225</v>
+        <v>13.95167726939298</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.3040456642072235</v>
+        <v>1.234844571663057</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.1578583735868139</v>
+        <v>94.52794024248088</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6477</v>
+        <v>6208</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>安集</t>
+          <t>日揚</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>286.4502613287738</v>
+        <v>291.3313815875944</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>33.95</v>
+        <v>81.7</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>43.37166705898985</v>
+        <v>44.02708707802903</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>16.97922797804473</v>
+        <v>16.66578478987826</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.2215247056356196</v>
+        <v>0.9407008158382956</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.5107340494142445</v>
+        <v>0.2488588667002425</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6415</v>
+        <v>6197</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>矽力*-KY</t>
+          <t>佳必琪</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>283.6435242083139</v>
+        <v>290.7420034366085</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>465</v>
+        <v>309</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>49.33236413881773</v>
+        <v>49.27257213589504</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>20.58562664275986</v>
+        <v>19.20985592526348</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.6589164054743736</v>
+        <v>0.9648127531215788</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>6.783230712566947</v>
+        <v>0.9338417424029366</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6209</v>
+        <v>6272</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>今國光</t>
+          <t>驊陞</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>272.9438452146628</v>
+        <v>287.9809485687836</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>74</v>
+        <v>25.1</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>51.72679550536951</v>
+        <v>39.49926573118158</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>16.91662821541473</v>
+        <v>40.31524748927225</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.9282442957113188</v>
+        <v>0.3040456642072235</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>1.402312812022273</v>
+        <v>0.1578583735868139</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6230</v>
+        <v>6443</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>尼得科超眾</t>
+          <t>元晶</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>262.8933382391858</v>
+        <v>281.8605787463625</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>110</v>
+        <v>27.05</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>41.08825921834021</v>
+        <v>43.89761042925628</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>30.74406490376641</v>
+        <v>28.15759170920897</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.5781209613052208</v>
+        <v>0.7605653134049977</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.4429766073275809</v>
+        <v>0.4570613136076846</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6443</v>
+        <v>6239</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>元晶</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>251.8605787463625</v>
+        <v>279.235622848787</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>27.05</v>
+        <v>288.5</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>43.89761042925628</v>
+        <v>52.97887863304339</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>28.15759170920897</v>
+        <v>16.93969890618489</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.7605653134049977</v>
+        <v>0.3712256943201117</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.4570613136076846</v>
+        <v>3.553993633587414</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6176</v>
+        <v>6442</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>瑞儀</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>243.100983376216</v>
+        <v>275.8860407547625</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>82.3</v>
+        <v>1425</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>38.46487597265871</v>
+        <v>51.16117003979465</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>21.68537825760686</v>
+        <v>23.67396318234185</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.7036948869608187</v>
+        <v>1.204091036502204</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.0270765751039372</v>
+        <v>39.23105388440921</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6205</v>
+        <v>6176</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>詮欣</t>
+          <t>瑞儀</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>239.1524623542154</v>
+        <v>273.1009833762159</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>61.5</v>
+        <v>82.3</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>46.45508190768687</v>
+        <v>38.46487597265871</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>29.75215094360628</v>
+        <v>21.68537825760686</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.4889966154262554</v>
+        <v>0.7036948869608187</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>1.012582027457825</v>
+        <v>-0.0270765751039372</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6185</v>
+        <v>6230</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>幃翔</t>
+          <t>尼得科超眾</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>222.885131429598</v>
+        <v>262.8933382391858</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>13.7</v>
+        <v>110</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>42.6877721119601</v>
+        <v>41.08825921834021</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>11.59677679826853</v>
+        <v>30.74406490376641</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.5026616149427816</v>
+        <v>0.5781209613052208</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.0236661808038683</v>
+        <v>0.4429766073275809</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6170</v>
+        <v>6415</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>統振</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>217.6497984685856</v>
+        <v>243.6435242083139</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>46.75</v>
+        <v>465</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>40.77890060401315</v>
+        <v>49.33236413881773</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>35.72179169242083</v>
+        <v>20.58562664275986</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.661861197280782</v>
+        <v>0.6589164054743736</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.187081502455551</v>
+        <v>6.783230712566947</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6283</v>
+        <v>6209</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>淳安</t>
+          <t>今國光</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>208.5046970566998</v>
+        <v>232.9438452146628</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>20.15</v>
+        <v>74</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>35.31092862846783</v>
+        <v>51.72679550536951</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>37.15218989297408</v>
+        <v>16.91662821541473</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.8323686662273455</v>
+        <v>0.9282442957113188</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.0628677858006557</v>
+        <v>1.402312812022273</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6189</v>
+        <v>6185</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>豐藝</t>
+          <t>幃翔</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>201.1319985267957</v>
+        <v>222.885131429598</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>49.05</v>
+        <v>13.7</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>50.67352634775676</v>
+        <v>42.6877721119601</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>12.19694852122346</v>
+        <v>11.59677679826853</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>1.145919097776142</v>
+        <v>0.5026616149427816</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.3153184743380142</v>
+        <v>-0.0236661808038683</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6218</v>
+        <v>6170</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>豪勉</t>
+          <t>統振</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>200.3602628461556</v>
+        <v>217.6497984685856</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>36.1</v>
+        <v>46.75</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>56.54724414854483</v>
+        <v>40.77890060401315</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>12.02101610242847</v>
+        <v>35.72179169242083</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.7414174001576361</v>
+        <v>0.661861197280782</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.4270261059824491</v>
+        <v>0.187081502455551</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6167</v>
+        <v>6283</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>久正</t>
+          <t>淳安</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>187.6680419392304</v>
+        <v>208.5046970566998</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>10.6</v>
+        <v>20.15</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>44.20309361337731</v>
+        <v>35.31092862846783</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>22.00275520034725</v>
+        <v>37.15218989297408</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.3641089052041301</v>
+        <v>0.8323686662273455</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0452256904481102</v>
+        <v>0.0628677858006557</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3813,21 +3813,21 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6438</v>
+        <v>6218</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>迅得</t>
+          <t>豪勉</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>179.9651212431265</v>
+        <v>200.3602628461556</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>147</v>
+        <v>36.1</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,16 +3838,16 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>50.75119064629824</v>
+        <v>56.54724414854483</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>22.69980200634814</v>
+        <v>12.02101610242847</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.3696585347344731</v>
+        <v>0.7414174001576361</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>1.34823973745081</v>
+        <v>0.4270261059824491</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6198</v>
+        <v>6205</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>瑞築</t>
+          <t>詮欣</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>174.9873341557976</v>
+        <v>199.1524623542154</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>19.5</v>
+        <v>61.5</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>51.65137386098494</v>
+        <v>46.45508190768687</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>8.727524867207372</v>
+        <v>29.75215094360628</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.2155079676989056</v>
+        <v>0.4889966154262554</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,11 +3909,11 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.4388121450622013</v>
+        <v>1.012582027457825</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, hist_turn_positive, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3930,7 @@
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>163.1788798683914</v>
+        <v>193.1788798683914</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>39.95</v>
@@ -3972,21 +3972,21 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6201</v>
+        <v>6228</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>亞弘電</t>
+          <t>全譜</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>137.3786017942331</v>
+        <v>193.0968173881948</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>45.45</v>
+        <v>17.55</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>29.22608246598594</v>
+        <v>51.12407703518314</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>15.86518354650595</v>
+        <v>10.26916350645334</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.6357624002122155</v>
+        <v>1.672024406724134</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.4331030236711123</v>
+        <v>0.4135605846389678</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6210</v>
+        <v>6167</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>慶生</t>
+          <t>久正</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>136.6174210068478</v>
+        <v>187.6680419392304</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>17.05</v>
+        <v>10.6</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>49.11131091030587</v>
+        <v>44.20309361337731</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>14.89637987282742</v>
+        <v>22.00275520034725</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.9651835149133774</v>
+        <v>0.3641089052041301</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.2569601624107177</v>
+        <v>0.0452256904481102</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6235</v>
+        <v>6189</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>華孚</t>
+          <t>豐藝</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>96.75640038535536</v>
+        <v>181.1319985267957</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>39.75</v>
+        <v>49.05</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>51.11386746324438</v>
+        <v>50.67352634775676</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>14.18654942921434</v>
+        <v>12.19694852122346</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.3431481457556441</v>
+        <v>1.145919097776142</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.2829840148598264</v>
+        <v>0.3153184743380142</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6216</v>
+        <v>6438</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>居易</t>
+          <t>迅得</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>92.14896717171855</v>
+        <v>179.9651212431265</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>21.9</v>
+        <v>147</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>43.51445079833805</v>
+        <v>50.75119064629824</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>13.68004799884843</v>
+        <v>22.69980200634814</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.9975319181756408</v>
+        <v>0.3696585347344731</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,62 +4174,433 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.0326616722666913</v>
+        <v>1.34823973745081</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
+        <v>6198</v>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>瑞築</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>174.9873341557976</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>51.65137386098494</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>8.727524867207372</v>
+      </c>
+      <c r="J71" s="2" t="n">
+        <v>0.2155079676989056</v>
+      </c>
+      <c r="K71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N71" s="2" t="n">
+        <v>0.4388121450622013</v>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>macd_golden_cross, market_above_ma60, hist_turn_positive, above_ichimoku_cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>6233</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>旺玖</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>165.6092593287854</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>48.04640689254035</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>30.6112588544335</v>
+      </c>
+      <c r="J72" s="2" t="n">
+        <v>0.6623345041445429</v>
+      </c>
+      <c r="K72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N72" s="2" t="n">
+        <v>0.1508209022986544</v>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>6201</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>亞弘電</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>137.3786017942331</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>45.45</v>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>29.22608246598594</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>15.86518354650595</v>
+      </c>
+      <c r="J73" s="2" t="n">
+        <v>0.6357624002122155</v>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N73" s="2" t="n">
+        <v>-0.4331030236711123</v>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>6210</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>慶生</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>136.6174210068478</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>49.11131091030587</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>14.89637987282742</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>0.9651835149133774</v>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>0.2569601624107177</v>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>6216</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>居易</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>122.1489671717186</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>43.51445079833805</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>13.68004799884843</v>
+      </c>
+      <c r="J75" s="2" t="n">
+        <v>0.9975319181756408</v>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N75" s="2" t="n">
+        <v>0.0326616722666913</v>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>6222</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>立軒</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>118.2392456072611</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>51.16310915159138</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>16.04776659063952</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>2.52432492101957</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>-0.0834759897303574</v>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>6235</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>華孚</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>96.75640038535536</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>39.75</v>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>51.11386746324438</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>14.18654942921434</v>
+      </c>
+      <c r="J77" s="2" t="n">
+        <v>0.3431481457556441</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N77" s="2" t="n">
+        <v>0.2829840148598264</v>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
         <v>6203</v>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>海韻電</t>
         </is>
       </c>
-      <c r="C71" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D71" s="2" t="n">
+      <c r="C78" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D78" s="2" t="n">
         <v>91.27343946356822</v>
       </c>
-      <c r="E71" s="2" t="n">
+      <c r="E78" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H71" s="2" t="n">
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H78" s="2" t="n">
         <v>31.63659554236342</v>
       </c>
-      <c r="I71" s="2" t="n">
+      <c r="I78" s="2" t="n">
         <v>16.32956395134587</v>
       </c>
-      <c r="J71" s="2" t="n">
+      <c r="J78" s="2" t="n">
         <v>0.8303317927924019</v>
       </c>
-      <c r="K71" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L71" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M71" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N71" s="2" t="n">
+      <c r="K78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N78" s="2" t="n">
         <v>-0.4010030504976853</v>
       </c>
-      <c r="O71" s="2" t="inlineStr">
+      <c r="O78" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>